<commit_message>
cập nhật tài liệu elearning
</commit_message>
<xml_diff>
--- a/hrm/.plans/elearning-hoc-vien/chi-tiet-khoa-hoc/testcase.xlsx
+++ b/hrm/.plans/elearning-hoc-vien/chi-tiet-khoa-hoc/testcase.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O44"/>
+  <dimension ref="A1:O47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -599,7 +599,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Trang chi tiết khóa học: giới thiệu khóa, cho tham gia (ghi danh), xem tiêu chí hoàn thành, xem nội dung chương→bài và vào học, thảo luận/đánh giá. Khóa exam-mode (nhân viên) có khối bài thi.</t>
+          <t>Trang chi tiết khóa học: giới thiệu khóa, cho tham gia (ghi danh), xem tiêu chí hoàn thành, xem nội dung chương→bài và vào học, thảo luận/đánh giá. Khóa exam-mode có khối bài thi (học viên ngoài thi native trong elearning nếu khóa Public; nhân viên thi trên HRM).</t>
         </is>
       </c>
       <c r="C2" s="4" t="n"/>
@@ -652,7 +652,7 @@
       <c r="B4" s="3" t="inlineStr">
         <is>
           <t>► Khách chưa đăng nhập: bấm Tham gia/Học → yêu cầu đăng nhập.
-► Học viên ngoài + khóa exam-mode → bị chặn (chỉ dành cho nhân viên).
+► Học viên ngoài chỉ bị chặn khi khóa exam-mode KHÔNG công khai (khóa Public → thi native được).
 ► Không có quyền/khóa không tồn tại → khối lỗi.</t>
         </is>
       </c>
@@ -1935,7 +1935,7 @@
       <c r="B33" s="11" t="n"/>
       <c r="C33" s="12" t="inlineStr">
         <is>
-          <t>III. BÀI THI (EXAM-MODE)</t>
+          <t>III. BÀI THI (EXAM-MODE) — xem thêm tài liệu 'Luồng làm bài thi'</t>
         </is>
       </c>
       <c r="D33" s="4" t="n"/>
@@ -1959,7 +1959,7 @@
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>BÀI THI (EXAM-MODE)</t>
+          <t>BÀI THI (EXAM-MODE) — xem thêm tài liệu 'Luồng làm bài thi'</t>
         </is>
       </c>
       <c r="C34" s="14" t="inlineStr">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>Nhân viên đã ghi danh khóa exam-mode</t>
+          <t>Đã ghi danh khóa exam-mode</t>
         </is>
       </c>
       <c r="G34" s="14" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="O34" s="14" t="inlineStr"/>
     </row>
-    <row r="35" ht="34" customHeight="1">
+    <row r="35" ht="38" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
         <is>
           <t>Chi tiết khóa</t>
@@ -2028,7 +2028,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>BÀI THI (EXAM-MODE)</t>
+          <t>BÀI THI (EXAM-MODE) — xem thêm tài liệu 'Luồng làm bài thi'</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Học viên ngoài bị chặn exam-mode</t>
+          <t>Học viên ngoài — khóa exam-mode Public (thi native)</t>
         </is>
       </c>
       <c r="E35" s="13" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Học viên ngoài, khóa exam-mode</t>
+          <t>Học viên ngoài, khóa exam-mode CÔNG KHAI, đã tham gia</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>- Ẩn nút; hiện 'Khoá học này hoàn thành bằng bài thi trên hệ thống nội bộ — chỉ dành cho nhân viên...'</t>
+          <t>- Hiện khối bài thi + 'Bạn làm bài thi trực tiếp trên hệ thống học trực tuyến.' + nút 'Làm đề thi' (KHÔNG bị chặn)</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="O35" s="3" t="inlineStr"/>
     </row>
-    <row r="36" ht="30" customHeight="1">
+    <row r="36" ht="45" customHeight="1">
       <c r="A36" s="14" t="inlineStr">
         <is>
           <t>Chi tiết khóa</t>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="B36" s="14" t="inlineStr">
         <is>
-          <t>BÀI THI (EXAM-MODE)</t>
+          <t>BÀI THI (EXAM-MODE) — xem thêm tài liệu 'Luồng làm bài thi'</t>
         </is>
       </c>
       <c r="C36" s="14" t="inlineStr">
@@ -2107,22 +2107,22 @@
       </c>
       <c r="D36" s="14" t="inlineStr">
         <is>
-          <t>Chưa đủ điều kiện thi</t>
+          <t>Học viên ngoài — khóa exam-mode KHÔNG Public (bị chặn)</t>
         </is>
       </c>
       <c r="E36" s="15" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="F36" s="14" t="inlineStr">
         <is>
-          <t>Chưa hoàn thành đủ % bài học</t>
+          <t>Học viên ngoài, khóa exam-mode KHÔNG công khai</t>
         </is>
       </c>
       <c r="G36" s="14" t="inlineStr">
         <is>
-          <t>1. Xem nút 'Làm đề thi'</t>
+          <t>1. Xem card ghi danh</t>
         </is>
       </c>
       <c r="H36" s="14" t="inlineStr">
@@ -2132,12 +2132,12 @@
       </c>
       <c r="I36" s="14" t="inlineStr">
         <is>
-          <t>- Nút bị vô hiệu + 'Cần hoàn thành ≥ {X}% bài học để được thi.'</t>
+          <t>- Ẩn nút; banner 'Khoá học này hoàn thành bằng bài thi trên hệ thống nội bộ — chỉ dành cho nhân viên, không áp dụng cho học viên ngoài.'</t>
         </is>
       </c>
       <c r="J36" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BR-04</t>
         </is>
       </c>
       <c r="K36" s="14" t="inlineStr"/>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>BÀI THI (EXAM-MODE)</t>
+          <t>BÀI THI (EXAM-MODE) — xem thêm tài liệu 'Luồng làm bài thi'</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Làm đề thi deep-link HRM</t>
+          <t>Nhân viên — text nơi thi HRM</t>
         </is>
       </c>
       <c r="E37" s="13" t="inlineStr">
@@ -2186,12 +2186,12 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Đủ điều kiện thi</t>
+          <t>Nhân viên, khóa exam-mode, đã tham gia</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>1. Bấm 'Làm đề thi'</t>
+          <t>1. Xem khối bài thi</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>- Chuyển sang hệ thống HRM (kèm link quay lại)</t>
+          <t>- Dòng 'Bài thi sẽ thực hiện ở phân hệ Đào tạo (HRM).'</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
@@ -2235,7 +2235,7 @@
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>BÀI THI (EXAM-MODE)</t>
+          <t>BÀI THI (EXAM-MODE) — xem thêm tài liệu 'Luồng làm bài thi'</t>
         </is>
       </c>
       <c r="C38" s="14" t="inlineStr">
@@ -2245,22 +2245,22 @@
       </c>
       <c r="D38" s="14" t="inlineStr">
         <is>
-          <t>Xem lịch sử thi</t>
+          <t>Chưa đủ điều kiện thi</t>
         </is>
       </c>
       <c r="E38" s="15" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="F38" s="14" t="inlineStr">
         <is>
-          <t>Đã thi ≥1 lần</t>
+          <t>Chưa hoàn thành đủ % bài học</t>
         </is>
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
-          <t>1. Bấm 'Lịch sử thi ({n})'</t>
+          <t>1. Xem nút 'Làm đề thi'</t>
         </is>
       </c>
       <c r="H38" s="14" t="inlineStr">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="I38" s="14" t="inlineStr">
         <is>
-          <t>- Mở popup lịch sử các lượt thi</t>
+          <t>- Nút bị vô hiệu + 'Cần hoàn thành ≥ {X}% bài học để được thi.'</t>
         </is>
       </c>
       <c r="J38" s="14" t="inlineStr">
@@ -2296,380 +2296,586 @@
       </c>
       <c r="O38" s="14" t="inlineStr"/>
     </row>
-    <row r="39" ht="26" customHeight="1">
-      <c r="A39" s="11" t="n"/>
-      <c r="B39" s="11" t="n"/>
-      <c r="C39" s="12" t="inlineStr">
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Chi tiết khóa</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>BÀI THI (EXAM-MODE) — xem thêm tài liệu 'Luồng làm bài thi'</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>TC_03.006</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Làm đề thi — học viên ngoài (native)</t>
+        </is>
+      </c>
+      <c r="E39" s="13" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Học viên ngoài đủ điều kiện</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>1. Bấm 'Làm đề thi'</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>- Mở màn thi native trong elearning (/khoa-hoc/:slug/thi)</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>BR-04</t>
+        </is>
+      </c>
+      <c r="K39" s="3" t="inlineStr"/>
+      <c r="L39" s="3" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M39" s="3" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N39" s="3" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="O39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>Chi tiết khóa</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>BÀI THI (EXAM-MODE) — xem thêm tài liệu 'Luồng làm bài thi'</t>
+        </is>
+      </c>
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>TC_03.007</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr">
+        <is>
+          <t>Làm đề thi — nhân viên (HRM)</t>
+        </is>
+      </c>
+      <c r="E40" s="15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F40" s="14" t="inlineStr">
+        <is>
+          <t>Nhân viên đủ điều kiện</t>
+        </is>
+      </c>
+      <c r="G40" s="14" t="inlineStr">
+        <is>
+          <t>1. Bấm 'Làm đề thi'</t>
+        </is>
+      </c>
+      <c r="H40" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I40" s="14" t="inlineStr">
+        <is>
+          <t>- Chuyển sang hệ thống HRM (kèm link quay lại)</t>
+        </is>
+      </c>
+      <c r="J40" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K40" s="14" t="inlineStr"/>
+      <c r="L40" s="14" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M40" s="14" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N40" s="14" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="O40" s="14" t="inlineStr"/>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Chi tiết khóa</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>BÀI THI (EXAM-MODE) — xem thêm tài liệu 'Luồng làm bài thi'</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>TC_03.008</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Xem lịch sử thi</t>
+        </is>
+      </c>
+      <c r="E41" s="13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Đã thi ≥1 lần</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>1. Bấm 'Lịch sử thi ({n})'</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>- Mở popup 'Lịch sử thi' (Lần/Thời gian/Đề thi/Điểm/Kết quả)</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K41" s="3" t="inlineStr"/>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M41" s="3" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N41" s="3" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="O41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="26" customHeight="1">
+      <c r="A42" s="11" t="n"/>
+      <c r="B42" s="11" t="n"/>
+      <c r="C42" s="12" t="inlineStr">
         <is>
           <t>IV. THẢO LUẬN</t>
         </is>
       </c>
-      <c r="D39" s="4" t="n"/>
-      <c r="E39" s="4" t="n"/>
-      <c r="F39" s="4" t="n"/>
-      <c r="G39" s="4" t="n"/>
-      <c r="H39" s="4" t="n"/>
-      <c r="I39" s="4" t="n"/>
-      <c r="J39" s="4" t="n"/>
-      <c r="K39" s="4" t="n"/>
-      <c r="L39" s="4" t="n"/>
-      <c r="M39" s="4" t="n"/>
-      <c r="N39" s="4" t="n"/>
-      <c r="O39" s="5" t="n"/>
-    </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="3" t="inlineStr">
+      <c r="D42" s="4" t="n"/>
+      <c r="E42" s="4" t="n"/>
+      <c r="F42" s="4" t="n"/>
+      <c r="G42" s="4" t="n"/>
+      <c r="H42" s="4" t="n"/>
+      <c r="I42" s="4" t="n"/>
+      <c r="J42" s="4" t="n"/>
+      <c r="K42" s="4" t="n"/>
+      <c r="L42" s="4" t="n"/>
+      <c r="M42" s="4" t="n"/>
+      <c r="N42" s="4" t="n"/>
+      <c r="O42" s="5" t="n"/>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="14" t="inlineStr">
         <is>
           <t>Chi tiết khóa</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="B43" s="14" t="inlineStr">
         <is>
           <t>THẢO LUẬN</t>
         </is>
       </c>
-      <c r="C40" s="3" t="inlineStr">
+      <c r="C43" s="14" t="inlineStr">
         <is>
           <t>TC_04.001</t>
         </is>
       </c>
-      <c r="D40" s="3" t="inlineStr">
+      <c r="D43" s="14" t="inlineStr">
         <is>
           <t>Gửi bình luận + đánh giá</t>
         </is>
       </c>
-      <c r="E40" s="13" t="inlineStr">
+      <c r="E43" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F40" s="3" t="inlineStr">
+      <c r="F43" s="14" t="inlineStr">
         <is>
           <t>Đã đăng nhập, tab Thảo luận</t>
         </is>
       </c>
-      <c r="G40" s="3" t="inlineStr">
+      <c r="G43" s="14" t="inlineStr">
         <is>
           <t>1. Chọn 'Đánh giá' = 5 - Rất tốt
 2. Nhập 'Nội dung'
 3. Bấm 'Gửi'</t>
         </is>
       </c>
-      <c r="H40" s="3" t="inlineStr">
+      <c r="H43" s="14" t="inlineStr">
         <is>
           <t>5 sao + nội dung</t>
         </is>
       </c>
-      <c r="I40" s="3" t="inlineStr">
+      <c r="I43" s="14" t="inlineStr">
         <is>
           <t>- Toast 'Đã gửi bình luận', bình luận xuất hiện</t>
         </is>
       </c>
-      <c r="J40" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K40" s="3" t="inlineStr"/>
-      <c r="L40" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M40" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N40" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="O40" s="3" t="inlineStr"/>
-    </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="14" t="inlineStr">
+      <c r="J43" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K43" s="14" t="inlineStr"/>
+      <c r="L43" s="14" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M43" s="14" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N43" s="14" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="O43" s="14" t="inlineStr"/>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>Chi tiết khóa</t>
         </is>
       </c>
-      <c r="B41" s="14" t="inlineStr">
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>THẢO LUẬN</t>
         </is>
       </c>
-      <c r="C41" s="14" t="inlineStr">
+      <c r="C44" s="3" t="inlineStr">
         <is>
           <t>TC_04.002</t>
         </is>
       </c>
-      <c r="D41" s="14" t="inlineStr">
+      <c r="D44" s="3" t="inlineStr">
         <is>
           <t>Gửi bình luận trống</t>
         </is>
       </c>
-      <c r="E41" s="15" t="inlineStr">
+      <c r="E44" s="13" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F41" s="14" t="inlineStr">
+      <c r="F44" s="3" t="inlineStr">
         <is>
           <t>Tab Thảo luận</t>
         </is>
       </c>
-      <c r="G41" s="14" t="inlineStr">
+      <c r="G44" s="3" t="inlineStr">
         <is>
           <t>1. Để trống 'Nội dung'
 2. Bấm 'Gửi'</t>
         </is>
       </c>
-      <c r="H41" s="14" t="inlineStr">
+      <c r="H44" s="3" t="inlineStr">
         <is>
           <t>(trống)</t>
         </is>
       </c>
-      <c r="I41" s="14" t="inlineStr">
+      <c r="I44" s="3" t="inlineStr">
         <is>
           <t>- Toast 'Vui lòng nhập nội dung bình luận'</t>
         </is>
       </c>
-      <c r="J41" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K41" s="14" t="inlineStr"/>
-      <c r="L41" s="14" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M41" s="14" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N41" s="14" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="O41" s="14" t="inlineStr"/>
-    </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="3" t="inlineStr">
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr"/>
+      <c r="L44" s="3" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M44" s="3" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N44" s="3" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="O44" s="3" t="inlineStr"/>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="14" t="inlineStr">
         <is>
           <t>Chi tiết khóa</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr">
+      <c r="B45" s="14" t="inlineStr">
         <is>
           <t>THẢO LUẬN</t>
         </is>
       </c>
-      <c r="C42" s="3" t="inlineStr">
+      <c r="C45" s="14" t="inlineStr">
         <is>
           <t>TC_04.003</t>
         </is>
       </c>
-      <c r="D42" s="3" t="inlineStr">
+      <c r="D45" s="14" t="inlineStr">
         <is>
           <t>Bình luận khi chưa đăng nhập</t>
         </is>
       </c>
-      <c r="E42" s="13" t="inlineStr">
+      <c r="E45" s="15" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F42" s="3" t="inlineStr">
+      <c r="F45" s="14" t="inlineStr">
         <is>
           <t>Chưa đăng nhập</t>
         </is>
       </c>
-      <c r="G42" s="3" t="inlineStr">
+      <c r="G45" s="14" t="inlineStr">
         <is>
           <t>1. Bấm 'Gửi' bình luận</t>
         </is>
       </c>
-      <c r="H42" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I42" s="3" t="inlineStr">
+      <c r="H45" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I45" s="14" t="inlineStr">
         <is>
           <t>- Chuyển sang trang đăng nhập</t>
         </is>
       </c>
-      <c r="J42" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K42" s="3" t="inlineStr"/>
-      <c r="L42" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M42" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N42" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="O42" s="3" t="inlineStr"/>
-    </row>
-    <row r="43" ht="35" customHeight="1">
-      <c r="A43" s="14" t="inlineStr">
+      <c r="J45" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K45" s="14" t="inlineStr"/>
+      <c r="L45" s="14" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M45" s="14" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N45" s="14" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="O45" s="14" t="inlineStr"/>
+    </row>
+    <row r="46" ht="35" customHeight="1">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>Chi tiết khóa</t>
         </is>
       </c>
-      <c r="B43" s="14" t="inlineStr">
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t>THẢO LUẬN</t>
         </is>
       </c>
-      <c r="C43" s="14" t="inlineStr">
+      <c r="C46" s="3" t="inlineStr">
         <is>
           <t>TC_04.004</t>
         </is>
       </c>
-      <c r="D43" s="14" t="inlineStr">
+      <c r="D46" s="3" t="inlineStr">
         <is>
           <t>Trả lời / Thích / Báo cáo</t>
         </is>
       </c>
-      <c r="E43" s="15" t="inlineStr">
+      <c r="E46" s="13" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F43" s="14" t="inlineStr">
+      <c r="F46" s="3" t="inlineStr">
         <is>
           <t>Có bình luận sẵn</t>
         </is>
       </c>
-      <c r="G43" s="14" t="inlineStr">
+      <c r="G46" s="3" t="inlineStr">
         <is>
           <t>1. Bấm 'Trả lời' / 'Thích' / 'Báo cáo' một bình luận</t>
         </is>
       </c>
-      <c r="H43" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I43" s="14" t="inlineStr">
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
         <is>
           <t>- Trả lời: mở ô 'Viết câu trả lời...'; Báo cáo: popup 'Báo cáo bình luận' (Spam/Nội dung không phù hợp/...)</t>
         </is>
       </c>
-      <c r="J43" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K43" s="14" t="inlineStr"/>
-      <c r="L43" s="14" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M43" s="14" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N43" s="14" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="O43" s="14" t="inlineStr"/>
-    </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="3" t="inlineStr">
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr"/>
+      <c r="L46" s="3" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M46" s="3" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N46" s="3" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="O46" s="3" t="inlineStr"/>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="14" t="inlineStr">
         <is>
           <t>Chi tiết khóa</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr">
+      <c r="B47" s="14" t="inlineStr">
         <is>
           <t>THẢO LUẬN</t>
         </is>
       </c>
-      <c r="C44" s="3" t="inlineStr">
+      <c r="C47" s="14" t="inlineStr">
         <is>
           <t>TC_04.005</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr">
+      <c r="D47" s="14" t="inlineStr">
         <is>
           <t>Trang thảo luận riêng + lọc sao</t>
         </is>
       </c>
-      <c r="E44" s="13" t="inlineStr">
+      <c r="E47" s="15" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F44" s="3" t="inlineStr">
+      <c r="F47" s="14" t="inlineStr">
         <is>
           <t>Khóa có nhiều đánh giá</t>
         </is>
       </c>
-      <c r="G44" s="3" t="inlineStr">
+      <c r="G47" s="14" t="inlineStr">
         <is>
           <t>1. Mở /khoa-hoc/:slug/thao-luan
 2. Bấm lọc '5 sao'</t>
         </is>
       </c>
-      <c r="H44" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I44" s="3" t="inlineStr">
+      <c r="H47" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I47" s="14" t="inlineStr">
         <is>
           <t>- Hiện tổng đánh giá {avg}/5, các thanh sao; lọc theo '5 sao' đúng</t>
         </is>
       </c>
-      <c r="J44" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K44" s="3" t="inlineStr"/>
-      <c r="L44" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="M44" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="N44" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
-        </is>
-      </c>
-      <c r="O44" s="3" t="inlineStr"/>
+      <c r="J47" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K47" s="14" t="inlineStr"/>
+      <c r="L47" s="14" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="M47" s="14" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="N47" s="14" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="O47" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="26">
     <mergeCell ref="B4:O4"/>
-    <mergeCell ref="C39:O39"/>
     <mergeCell ref="B7:O7"/>
     <mergeCell ref="B3:O3"/>
     <mergeCell ref="I12:K12"/>
@@ -2679,6 +2885,7 @@
     <mergeCell ref="C18:O18"/>
     <mergeCell ref="C33:O33"/>
     <mergeCell ref="C24:O24"/>
+    <mergeCell ref="C42:O42"/>
     <mergeCell ref="B1:O1"/>
     <mergeCell ref="B8:O8"/>
     <mergeCell ref="L13:O13"/>
@@ -2696,7 +2903,7 @@
     <mergeCell ref="B5:O5"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="L18:N145" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L18:N148" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Passed,Failed,Pending,Not Executed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>